<commit_message>
Improve the analyzer for MYP gradebooks and teacher feedback.
Add criterion scatter pickers, keep extra columns like attendance, clarify chart titles, and ship generic Criterion A–D templates plus three demo classes with clear patterns.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/subject-gradebook-template.xlsx
+++ b/templates/subject-gradebook-template.xlsx
@@ -397,9 +397,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:X13"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
@@ -420,6 +420,9 @@
     <col min="19" max="19" width="14.83203125" customWidth="1"/>
     <col min="20" max="20" width="14.83203125" customWidth="1"/>
     <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,70 +489,88 @@
       <c r="U1" t="str">
         <v/>
       </c>
+      <c r="V1" t="str">
+        <v/>
+      </c>
+      <c r="W1" t="str">
+        <v/>
+      </c>
+      <c r="X1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>Student Name</v>
       </c>
       <c r="B2" t="str">
-        <v>Knowing and Understanding</v>
+        <v>Criterion A</v>
       </c>
       <c r="C2" t="str">
-        <v>Investigating Patterns</v>
+        <v>Criterion B</v>
       </c>
       <c r="D2" t="str">
-        <v>Communicating</v>
+        <v>Criterion C</v>
       </c>
       <c r="E2" t="str">
-        <v>Applying Mathematics in Real-World Contexts</v>
+        <v>Criterion D</v>
       </c>
       <c r="F2" t="str">
-        <v>Knowing and Understanding</v>
+        <v>Criterion A</v>
       </c>
       <c r="G2" t="str">
-        <v>Investigating Patterns</v>
+        <v>Criterion B</v>
       </c>
       <c r="H2" t="str">
-        <v>Communicating</v>
+        <v>Criterion C</v>
       </c>
       <c r="I2" t="str">
-        <v>Applying Mathematics in Real-World Contexts</v>
+        <v>Criterion D</v>
       </c>
       <c r="J2" t="str">
-        <v>Knowing and Understanding</v>
+        <v>Criterion A</v>
       </c>
       <c r="K2" t="str">
-        <v>Investigating Patterns</v>
+        <v>Criterion B</v>
       </c>
       <c r="L2" t="str">
-        <v>Communicating</v>
+        <v>Criterion C</v>
       </c>
       <c r="M2" t="str">
-        <v>Applying Mathematics in Real-World Contexts</v>
+        <v>Criterion D</v>
       </c>
       <c r="N2" t="str">
-        <v>Knowing and Understanding</v>
+        <v>Criterion A</v>
       </c>
       <c r="O2" t="str">
-        <v>Investigating Patterns</v>
+        <v>Criterion B</v>
       </c>
       <c r="P2" t="str">
-        <v>Communicating</v>
+        <v>Criterion C</v>
       </c>
       <c r="Q2" t="str">
-        <v>Applying Mathematics in Real-World Contexts</v>
+        <v>Criterion D</v>
       </c>
       <c r="R2" t="str">
-        <v>Knowing and Understanding</v>
+        <v>Criterion A</v>
       </c>
       <c r="S2" t="str">
-        <v>Investigating Patterns</v>
+        <v>Criterion B</v>
       </c>
       <c r="T2" t="str">
-        <v>Communicating</v>
+        <v>Criterion C</v>
       </c>
       <c r="U2" t="str">
-        <v>Applying Mathematics in Real-World Contexts</v>
+        <v>Criterion D</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Attendance %</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Homework %</v>
+      </c>
+      <c r="X2" t="str">
+        <v>EAL</v>
       </c>
     </row>
     <row r="3">
@@ -616,6 +637,15 @@
       <c r="U3" t="str">
         <v>4</v>
       </c>
+      <c r="V3">
+        <v>96</v>
+      </c>
+      <c r="W3">
+        <v>100</v>
+      </c>
+      <c r="X3" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -681,6 +711,15 @@
       <c r="U4" t="str">
         <v>7</v>
       </c>
+      <c r="V4">
+        <v>94</v>
+      </c>
+      <c r="W4">
+        <v>88</v>
+      </c>
+      <c r="X4" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -746,6 +785,15 @@
       <c r="U5" t="str">
         <v>7</v>
       </c>
+      <c r="V5">
+        <v>98</v>
+      </c>
+      <c r="W5">
+        <v>92</v>
+      </c>
+      <c r="X5" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -811,6 +859,15 @@
       <c r="U6" t="str">
         <v>3</v>
       </c>
+      <c r="V6">
+        <v>91</v>
+      </c>
+      <c r="W6">
+        <v>80</v>
+      </c>
+      <c r="X6" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -876,6 +933,15 @@
       <c r="U7" t="str">
         <v>5</v>
       </c>
+      <c r="V7">
+        <v>95</v>
+      </c>
+      <c r="W7">
+        <v>90</v>
+      </c>
+      <c r="X7" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -941,6 +1007,15 @@
       <c r="U8" t="str">
         <v>7</v>
       </c>
+      <c r="V8">
+        <v>95</v>
+      </c>
+      <c r="W8">
+        <v>90</v>
+      </c>
+      <c r="X8" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1006,6 +1081,15 @@
       <c r="U9" t="str">
         <v>6</v>
       </c>
+      <c r="V9">
+        <v>95</v>
+      </c>
+      <c r="W9">
+        <v>90</v>
+      </c>
+      <c r="X9" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1071,6 +1155,15 @@
       <c r="U10" t="str">
         <v>3</v>
       </c>
+      <c r="V10">
+        <v>95</v>
+      </c>
+      <c r="W10">
+        <v>90</v>
+      </c>
+      <c r="X10" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1136,6 +1229,15 @@
       <c r="U11" t="str">
         <v>-</v>
       </c>
+      <c r="V11">
+        <v>95</v>
+      </c>
+      <c r="W11">
+        <v>90</v>
+      </c>
+      <c r="X11" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1201,6 +1303,15 @@
       <c r="U12" t="str">
         <v/>
       </c>
+      <c r="V12">
+        <v>95</v>
+      </c>
+      <c r="W12">
+        <v>90</v>
+      </c>
+      <c r="X12" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1266,17 +1377,19 @@
       <c r="U13" t="str">
         <v/>
       </c>
+      <c r="V13">
+        <v>95</v>
+      </c>
+      <c r="W13">
+        <v>90</v>
+      </c>
+      <c r="X13" t="str">
+        <v>No</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="N1:Q1"/>
-    <mergeCell ref="R1:U1"/>
-  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>